<commit_message>
docs: regenerate the output report, and point the README at the real PDFs
The output report in submission/ was generated on 5 September and predated the
re-seed; the index now holds 44 detections and 38 alerts, so the attached
artefact no longer matched what the platform would show a reviewer. Regenerated
from the live index.

The submission links table still told the reader to export HLD.md and
PRESENTATION.md themselves. Both PDFs exist now, so it names them.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission/sentinel_output_report.xlsx
+++ b/submission/sentinel_output_report.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detections" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detections'!$A$1:$M$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detections'!$A$1:$M$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-05 10:51:14</t>
+          <t>2026-09-11 09:38:27</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M63"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -687,54 +687,54 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>73.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F2" s="8" t="n">
-        <v>22.217</v>
+        <v>23.035</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 05:42:50 UTC</t>
         </is>
       </c>
       <c r="J2" s="8" t="n">
-        <v>1040</v>
+        <v>2000</v>
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t2</t>
+          <t>cam13-GJ03CJ6081-2</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ01AB1234_20260905_104513_929370.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
@@ -746,54 +746,54 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam12</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>22.217</v>
+        <v>23.1645</v>
       </c>
       <c r="G3" t="n">
-        <v>70.79000000000001</v>
+        <v>72.581</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:58:50 UTC</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>4280</v>
+        <v>3000</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>cam17-p1-t3</t>
+          <t>cam12-GJ18DH2745-3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ01AB1234_20260905_104617_690855.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -805,54 +805,54 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>97.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam03</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>03 O.N.G.C. Office</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F4" s="8" t="n">
-        <v>22.217</v>
+        <v>23.0587</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.53100000000001</v>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>ONGC Office, Chandkheda, Ahmedabad</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:54:50 UTC</t>
         </is>
       </c>
       <c r="J4" s="8" t="n">
-        <v>8720</v>
+        <v>3000</v>
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t4</t>
+          <t>cam03-MH12QP5837-3</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ18CD5678_20260905_104722_815397.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
       <c r="M4" s="8" t="inlineStr">
@@ -864,54 +864,54 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>22.217</v>
+        <v>23.0587</v>
       </c>
       <c r="G5" t="n">
-        <v>70.79000000000001</v>
+        <v>72.5806</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:43:50 UTC</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>13160</v>
+        <v>2000</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>cam17-p1-t5</t>
+          <t>cam01-RJ14SL3926-2</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ05JV7219_20260905_104746_554953.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -923,54 +923,54 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>97.3</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam02</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>02 Janpath</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>22.217</v>
+        <v>23.0299</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.57129999999999</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:41:50 UTC</t>
         </is>
       </c>
       <c r="J6" s="8" t="n">
-        <v>17480</v>
+        <v>4000</v>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t6</t>
+          <t>cam02-GJ01KA7392-4</t>
         </is>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_MH12DE1433_20260905_104817_152931.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -982,54 +982,54 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>22.217</v>
+        <v>23.0999</v>
       </c>
       <c r="G7" t="n">
-        <v>70.79000000000001</v>
+        <v>72.5814</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:40:50 UTC</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>21920</v>
+        <v>2000</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>cam17-p1-t8</t>
+          <t>cam05-GJ18DH2745-2</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>/evidence/cam17_RJ14GH9012_20260905_104850_322066.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1041,54 +1041,54 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>GJ27XY4455</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>98.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam14</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>14 Delight RLVD</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F8" s="8" t="n">
-        <v>22.217</v>
+        <v>23.047</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.58799999999999</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:42:58 UTC</t>
+          <t>2026-09-11 04:36:50 UTC</t>
         </is>
       </c>
       <c r="J8" s="8" t="n">
-        <v>26360</v>
+        <v>2000</v>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t9</t>
+          <t>cam14-MH12QP5837-2</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ27XY4455_20260905_104908_646162.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -1100,54 +1100,54 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>73.59999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>22.217</v>
+        <v>23.035</v>
       </c>
       <c r="G9" t="n">
-        <v>70.79000000000001</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:33:50 UTC</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1040</v>
+        <v>3000</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>cam17-p1-t2</t>
+          <t>cam13-GJ01KA7392-3</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ01AB1234_20260905_104803_533257.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
@@ -1167,46 +1167,46 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>22.217</v>
+        <v>23.0999</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.5814</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:31:50 UTC</t>
         </is>
       </c>
       <c r="J10" s="8" t="n">
-        <v>4280</v>
+        <v>1000</v>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t3</t>
+          <t>cam05-RJ14SL3926-1</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ01AB1234_20260905_104828_413439.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -1218,54 +1218,54 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>97.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>22.217</v>
+        <v>23.035</v>
       </c>
       <c r="G11" t="n">
-        <v>70.79000000000001</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:25:50 UTC</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>8720</v>
+        <v>1000</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>cam17-p1-t4</t>
+          <t>cam13-MH12QP5837-1</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ18CD5678_20260905_104902_760081.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1277,54 +1277,54 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam18</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>18 Rajkot CCTV</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>22.217</v>
+        <v>22.3039</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>70.8022</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Rajkot City Surveillance</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:25:50 UTC</t>
         </is>
       </c>
       <c r="J12" s="8" t="n">
-        <v>13160</v>
+        <v>1000</v>
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t5</t>
+          <t>cam18-GJ03CJ6081-1</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_GJ05JV7219_20260905_104928_646884.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -1336,54 +1336,54 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>97.3</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam04</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>04 Paldi Circle</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>22.217</v>
+        <v>23.0104</v>
       </c>
       <c r="G13" t="n">
-        <v>70.79000000000001</v>
+        <v>72.5624</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:24:50 UTC</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>17480</v>
+        <v>2000</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>cam17-p1-t6</t>
+          <t>cam04-GJ01KA7392-2</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>/evidence/cam17_MH12DE1433_20260905_104950_253636.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>GJ27BG4108</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -1403,46 +1403,46 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>cam17</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>17 Rajkot Bus Port CCTV</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Municipal Corporation</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F14" s="8" t="n">
-        <v>22.217</v>
+        <v>23.0999</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>70.79000000000001</v>
+        <v>72.5814</v>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Rajkot Bus Port, Rajkot</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:25:34 UTC</t>
+          <t>2026-09-11 04:21:50 UTC</t>
         </is>
       </c>
       <c r="J14" s="8" t="n">
-        <v>21920</v>
+        <v>1000</v>
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>cam17-p1-t8</t>
+          <t>cam05-GJ27BG4108-1</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam17_RJ14GH9012_20260905_105013_834042.jpg</t>
+          <t>/evidence/cam16_GJ27BG4108_20260911_060753_475745.jpg</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -1454,54 +1454,54 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam02</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>02 Janpath</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>23.1645</v>
+        <v>23.0299</v>
       </c>
       <c r="G15" t="n">
-        <v>72.581</v>
+        <v>72.57129999999999</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:21:50 UTC</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>1040</v>
+        <v>1000</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>cam12-p1-t2</t>
+          <t>cam02-GJ18DH2745-1</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>/evidence/cam12_GJ01AB1234_20260905_104314_334376.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1513,7 +1513,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ27BG4108</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
@@ -1521,46 +1521,46 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam16</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>16 Visat P2</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F16" s="8" t="n">
-        <v>23.1645</v>
+        <v>23.101</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>72.581</v>
+        <v>72.583</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Visat Point 2, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:19:50 UTC</t>
         </is>
       </c>
       <c r="J16" s="8" t="n">
-        <v>4280</v>
+        <v>0</v>
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>cam12-p1-t3</t>
+          <t>cam16-GJ27BG4108-0</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam12_GJ01AB1234_20260905_104330_541419.jpg</t>
+          <t>/evidence/cam16_GJ27BG4108_20260911_060753_475745.jpg</t>
         </is>
       </c>
       <c r="M16" s="8" t="inlineStr">
@@ -1572,20 +1572,20 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>97.90000000000001</v>
+        <v>96</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam04</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>04 Paldi Circle</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1594,32 +1594,32 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>23.1645</v>
+        <v>23.0104</v>
       </c>
       <c r="G17" t="n">
-        <v>72.581</v>
+        <v>72.5624</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:15:50 UTC</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>8720</v>
+        <v>0</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>cam12-p1-t4</t>
+          <t>cam04-GJ18DH2745-0</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>/evidence/cam12_GJ18CD5678_20260905_104352_706013.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1631,20 +1631,20 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>94.5</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam14</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>14 Delight RLVD</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1653,32 +1653,32 @@
         </is>
       </c>
       <c r="F18" s="8" t="n">
-        <v>23.1645</v>
+        <v>23.047</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>72.581</v>
+        <v>72.58799999999999</v>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:12:50 UTC</t>
         </is>
       </c>
       <c r="J18" s="8" t="n">
-        <v>13160</v>
+        <v>1000</v>
       </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>cam12-p1-t5</t>
+          <t>cam14-GJ01KA7392-1</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam12_GJ05JV7219_20260905_104416_269777.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -1690,11 +1690,11 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1724,20 +1724,20 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:12:50 UTC</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>17480</v>
+        <v>0</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>cam12-p1-t6</t>
+          <t>cam12-RJ14SL3926-0</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>/evidence/cam12_MH12DE1433_20260905_104515_572532.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1749,54 +1749,54 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam15</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>15 Suvidha park</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F20" s="8" t="n">
-        <v>23.1645</v>
+        <v>23.081</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>72.581</v>
+        <v>72.529</v>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Suvidha Park, Ahmedabad</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:10:50 UTC</t>
         </is>
       </c>
       <c r="J20" s="8" t="n">
-        <v>21920</v>
+        <v>0</v>
       </c>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>cam12-p1-t8</t>
+          <t>cam15-MH12QP5837-0</t>
         </is>
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam12_RJ14GH9012_20260905_104704_562499.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
       <c r="M20" s="8" t="inlineStr">
@@ -1808,54 +1808,54 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>GJ27XY4455</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>98.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>cam12</t>
+          <t>cam17</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>12 Tri Mandir Adalaj Tollnaka</t>
+          <t>17 Rajkot Bus Port CCTV</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>Municipal Corporation</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>23.1645</v>
+        <v>22.217</v>
       </c>
       <c r="G21" t="n">
-        <v>72.581</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Tri Mandir, Adalaj Toll Naka</t>
+          <t>Rajkot Bus Port, Rajkot</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-05 09:21:34 UTC</t>
+          <t>2026-09-11 04:07:50 UTC</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>26360</v>
+        <v>0</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>cam12-p1-t9</t>
+          <t>cam17-GJ03CJ6081-0</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>/evidence/cam12_GJ27XY4455_20260905_104721_224378.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1867,20 +1867,20 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>73.59999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam01</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1889,32 +1889,32 @@
         </is>
       </c>
       <c r="F22" s="8" t="n">
-        <v>23.0999</v>
+        <v>23.0587</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>72.5814</v>
+        <v>72.5806</v>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-11 04:07:50 UTC</t>
         </is>
       </c>
       <c r="J22" s="8" t="n">
-        <v>1040</v>
+        <v>0</v>
       </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>cam05-p1-t2</t>
+          <t>cam01-GJ01KA7392-0</t>
         </is>
       </c>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam05_GJ01AB1234_20260905_104035_018668.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
       <c r="M22" s="8" t="inlineStr">
@@ -1926,20 +1926,20 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>RJ4E4555</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>100</v>
+        <v>78.5</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam12</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1948,32 +1948,32 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>23.0999</v>
+        <v>23.1645</v>
       </c>
       <c r="G23" t="n">
-        <v>72.5814</v>
+        <v>72.581</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 11:16:42 UTC</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>4280</v>
+        <v>7150</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>cam05-p1-t3</t>
+          <t>cam12-t2</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>/evidence/cam05_GJ01AB1234_20260905_104052_351361.jpg</t>
+          <t>/evidence/cam12_RJ4E4555_20260909_111641_637598.jpg</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1985,20 +1985,20 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>RJ3E4555</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>97.90000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam12</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -2007,32 +2007,32 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>23.0999</v>
+        <v>23.1645</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>72.5814</v>
+        <v>72.581</v>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 11:16:15 UTC</t>
         </is>
       </c>
       <c r="J24" s="8" t="n">
-        <v>8720</v>
+        <v>2150</v>
       </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>cam05-p1-t4</t>
+          <t>cam12-t1</t>
         </is>
       </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam05_GJ18CD5678_20260905_104115_705305.jpg</t>
+          <t>/evidence/cam12_RJ3E4555_20260909_111614_390210.jpg</t>
         </is>
       </c>
       <c r="M24" s="8" t="inlineStr">
@@ -2044,54 +2044,54 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>23.0999</v>
+        <v>23.035</v>
       </c>
       <c r="G25" t="n">
-        <v>72.5814</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 07:01:21 UTC</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>13160</v>
+        <v>2000</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>cam05-p1-t5</t>
+          <t>cam13-GJ03CJ6081-2</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>/evidence/cam05_GJ05JV7219_20260905_104140_188332.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2103,20 +2103,20 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>97.3</v>
+        <v>96</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam12</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -2125,32 +2125,32 @@
         </is>
       </c>
       <c r="F26" s="8" t="n">
-        <v>23.0999</v>
+        <v>23.1645</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>72.5814</v>
+        <v>72.581</v>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 06:17:21 UTC</t>
         </is>
       </c>
       <c r="J26" s="8" t="n">
-        <v>17480</v>
+        <v>3000</v>
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>cam05-p1-t6</t>
+          <t>cam12-GJ18DH2745-3</t>
         </is>
       </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam05_MH12DE1433_20260905_104237_879052.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
       <c r="M26" s="8" t="inlineStr">
@@ -2162,54 +2162,54 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam03</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>03 O.N.G.C. Office</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>23.0999</v>
+        <v>23.0587</v>
       </c>
       <c r="G27" t="n">
-        <v>72.5814</v>
+        <v>72.53100000000001</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>ONGC Office, Chandkheda, Ahmedabad</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 06:13:21 UTC</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>21920</v>
+        <v>3000</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>cam05-p1-t8</t>
+          <t>cam03-MH12QP5837-3</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>/evidence/cam05_RJ14GH9012_20260905_104255_299122.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2221,20 +2221,20 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>GJ27XY4455</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B28" s="8" t="n">
-        <v>98.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>cam05</t>
+          <t>cam01</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>05 Visat teen Rasta</t>
+          <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -2243,32 +2243,32 @@
         </is>
       </c>
       <c r="F28" s="8" t="n">
-        <v>23.0999</v>
+        <v>23.0587</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>72.5814</v>
+        <v>72.5806</v>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
+          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 09:07:34 UTC</t>
+          <t>2026-09-09 06:02:21 UTC</t>
         </is>
       </c>
       <c r="J28" s="8" t="n">
-        <v>26360</v>
+        <v>2000</v>
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>cam05-p1-t9</t>
+          <t>cam01-RJ14SL3926-2</t>
         </is>
       </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam05_GJ27XY4455_20260905_104304_974243.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
       <c r="M28" s="8" t="inlineStr">
@@ -2280,20 +2280,20 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>73.59999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam02</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>02 Janpath</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2302,32 +2302,32 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>23.081</v>
+        <v>23.0299</v>
       </c>
       <c r="G29" t="n">
-        <v>72.529</v>
+        <v>72.57129999999999</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 06:00:21 UTC</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>1040</v>
+        <v>4000</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>cam15-p1-t2</t>
+          <t>cam02-GJ01KA7392-4</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>/evidence/cam15_GJ01AB1234_20260905_103740_532697.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2339,54 +2339,54 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B30" s="8" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F30" s="8" t="n">
-        <v>23.081</v>
+        <v>23.0999</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>72.529</v>
+        <v>72.5814</v>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:59:21 UTC</t>
         </is>
       </c>
       <c r="J30" s="8" t="n">
-        <v>4280</v>
+        <v>2000</v>
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>cam15-p1-t3</t>
+          <t>cam05-GJ18DH2745-2</t>
         </is>
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam15_GJ01AB1234_20260905_103759_892171.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
       <c r="M30" s="8" t="inlineStr">
@@ -2398,54 +2398,54 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>97.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam14</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>14 Delight RLVD</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>23.081</v>
+        <v>23.047</v>
       </c>
       <c r="G31" t="n">
-        <v>72.529</v>
+        <v>72.58799999999999</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:55:21 UTC</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>8720</v>
+        <v>2000</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>cam15-p1-t4</t>
+          <t>cam14-MH12QP5837-2</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>/evidence/cam15_GJ18CD5678_20260905_103842_086627.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2457,20 +2457,20 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>94.5</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -2479,32 +2479,32 @@
         </is>
       </c>
       <c r="F32" s="8" t="n">
-        <v>23.081</v>
+        <v>23.035</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>72.529</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:52:21 UTC</t>
         </is>
       </c>
       <c r="J32" s="8" t="n">
-        <v>13160</v>
+        <v>3000</v>
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>cam15-p1-t5</t>
+          <t>cam13-GJ01KA7392-3</t>
         </is>
       </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam15_GJ05JV7219_20260905_103912_428558.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
       <c r="M32" s="8" t="inlineStr">
@@ -2516,54 +2516,54 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>23.081</v>
+        <v>23.0999</v>
       </c>
       <c r="G33" t="n">
-        <v>72.529</v>
+        <v>72.5814</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:50:21 UTC</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>17480</v>
+        <v>1000</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>cam15-p1-t6</t>
+          <t>cam05-RJ14SL3926-1</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>/evidence/cam15_MH12DE1433_20260905_103933_413406.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2575,7 +2575,7 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam18</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>18 Rajkot CCTV</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -2597,32 +2597,32 @@
         </is>
       </c>
       <c r="F34" s="8" t="n">
-        <v>23.081</v>
+        <v>22.3039</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>72.529</v>
+        <v>70.8022</v>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>Rajkot City Surveillance</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:44:21 UTC</t>
         </is>
       </c>
       <c r="J34" s="8" t="n">
-        <v>21920</v>
+        <v>1000</v>
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>cam15-p1-t8</t>
+          <t>cam18-GJ03CJ6081-1</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam15_RJ14GH9012_20260905_103956_209602.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
       <c r="M34" s="8" t="inlineStr">
@@ -2634,20 +2634,20 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>GJ27XY4455</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>98.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>cam15</t>
+          <t>cam13</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>15 Suvidha park</t>
+          <t>13 CN Vidhyalaya</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2656,32 +2656,32 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>23.081</v>
+        <v>23.035</v>
       </c>
       <c r="G35" t="n">
-        <v>72.529</v>
+        <v>72.54900000000001</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Suvidha Park, Ahmedabad</t>
+          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-05 08:58:34 UTC</t>
+          <t>2026-09-09 05:44:21 UTC</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>26360</v>
+        <v>1000</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>cam15-p1-t9</t>
+          <t>cam13-MH12QP5837-1</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>/evidence/cam15_GJ27XY4455_20260905_104010_442169.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2693,54 +2693,54 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>73.59999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam04</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>04 Paldi Circle</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F36" s="8" t="n">
-        <v>23.035</v>
+        <v>23.0104</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>72.54900000000001</v>
+        <v>72.5624</v>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:43:21 UTC</t>
         </is>
       </c>
       <c r="J36" s="8" t="n">
-        <v>1040</v>
+        <v>2000</v>
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>cam13-p1-t2</t>
+          <t>cam04-GJ01KA7392-2</t>
         </is>
       </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam13_GJ01AB1234_20260905_103452_101312.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
       <c r="M36" s="8" t="inlineStr">
@@ -2752,7 +2752,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ27BG4108</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2760,46 +2760,46 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam05</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>05 Visat teen Rasta</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>23.035</v>
+        <v>23.0999</v>
       </c>
       <c r="G37" t="n">
-        <v>72.54900000000001</v>
+        <v>72.5814</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:40:21 UTC</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>4280</v>
+        <v>1000</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>cam13-p1-t3</t>
+          <t>cam05-GJ27BG4108-1</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>/evidence/cam13_GJ01AB1234_20260905_103509_587491.jpg</t>
+          <t>/evidence/cam16_GJ27BG4108_20260909_072626_710757.jpg</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2811,20 +2811,20 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>97.90000000000001</v>
+        <v>96</v>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam02</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>02 Janpath</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2833,32 +2833,32 @@
         </is>
       </c>
       <c r="F38" s="8" t="n">
-        <v>23.035</v>
+        <v>23.0299</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>72.54900000000001</v>
+        <v>72.57129999999999</v>
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
       <c r="I38" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:40:21 UTC</t>
         </is>
       </c>
       <c r="J38" s="8" t="n">
-        <v>8720</v>
+        <v>1000</v>
       </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>cam13-p1-t4</t>
+          <t>cam02-GJ18DH2745-1</t>
         </is>
       </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam13_GJ18CD5678_20260905_103534_921717.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
       <c r="M38" s="8" t="inlineStr">
@@ -2870,20 +2870,20 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>GJ05JV7219</t>
+          <t>GJ27BG4108</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>94.5</v>
+        <v>100</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam16</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>16 Visat P2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2892,32 +2892,32 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>23.035</v>
+        <v>23.101</v>
       </c>
       <c r="G39" t="n">
-        <v>72.54900000000001</v>
+        <v>72.583</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Visat Point 2, Sabarmati, Ahmedabad</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:38:21 UTC</t>
         </is>
       </c>
       <c r="J39" t="n">
-        <v>13160</v>
+        <v>0</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>cam13-p1-t5</t>
+          <t>cam16-GJ27BG4108-0</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>/evidence/cam13_GJ05JV7219_20260905_103604_094126.jpg</t>
+          <t>/evidence/cam16_GJ27BG4108_20260909_072626_710757.jpg</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -2929,54 +2929,54 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>MH12DE1433</t>
+          <t>GJ18DH2745</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>97.3</v>
+        <v>96</v>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam04</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>04 Paldi Circle</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F40" s="8" t="n">
-        <v>23.035</v>
+        <v>23.0104</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>72.54900000000001</v>
+        <v>72.5624</v>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:34:21 UTC</t>
         </is>
       </c>
       <c r="J40" s="8" t="n">
-        <v>17480</v>
+        <v>0</v>
       </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>cam13-p1-t6</t>
+          <t>cam04-GJ18DH2745-0</t>
         </is>
       </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam13_MH12DE1433_20260905_103636_323535.jpg</t>
+          <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
       <c r="M40" s="8" t="inlineStr">
@@ -2988,54 +2988,54 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>RJ14GH9012</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam14</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>14 Delight RLVD</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>23.035</v>
+        <v>23.047</v>
       </c>
       <c r="G41" t="n">
-        <v>72.54900000000001</v>
+        <v>72.58799999999999</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:31:21 UTC</t>
         </is>
       </c>
       <c r="J41" t="n">
-        <v>21920</v>
+        <v>1000</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>cam13-p1-t8</t>
+          <t>cam14-GJ01KA7392-1</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>/evidence/cam13_RJ14GH9012_20260905_103701_025702.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3047,54 +3047,54 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>GJ27XY4455</t>
+          <t>RJ14SL3926</t>
         </is>
       </c>
       <c r="B42" s="8" t="n">
-        <v>98.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>cam13</t>
+          <t>cam12</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>13 CN Vidhyalaya</t>
+          <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>City Surveillance</t>
+          <t>Traffic Police</t>
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>23.035</v>
+        <v>23.1645</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>72.54900000000001</v>
+        <v>72.581</v>
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
+          <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:47:34 UTC</t>
+          <t>2026-09-09 05:31:21 UTC</t>
         </is>
       </c>
       <c r="J42" s="8" t="n">
-        <v>26360</v>
+        <v>0</v>
       </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>cam13-p1-t9</t>
+          <t>cam12-RJ14SL3926-0</t>
         </is>
       </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam13_GJ27XY4455_20260905_103714_049666.jpg</t>
+          <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
       <c r="M42" s="8" t="inlineStr">
@@ -3106,54 +3106,54 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>MH12QP5837</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>73.59999999999999</v>
+        <v>97</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>cam04</t>
+          <t>cam15</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>04 Paldi Circle</t>
+          <t>15 Suvidha park</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>City Surveillance</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>23.0104</v>
+        <v>23.081</v>
       </c>
       <c r="G43" t="n">
-        <v>72.5624</v>
+        <v>72.529</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
+          <t>Suvidha Park, Ahmedabad</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-05 08:40:34 UTC</t>
+          <t>2026-09-09 05:29:21 UTC</t>
         </is>
       </c>
       <c r="J43" t="n">
-        <v>1040</v>
+        <v>0</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>cam04-p1-t2</t>
+          <t>cam15-MH12QP5837-0</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>/evidence/cam04_GJ01AB1234_20260905_103226_382731.jpg</t>
+          <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3165,20 +3165,20 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>GJ01AB1234</t>
+          <t>GJ01KA7392</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>100</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>cam04</t>
+          <t>cam01</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>04 Paldi Circle</t>
+          <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -3187,32 +3187,32 @@
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>23.0104</v>
+        <v>23.0587</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>72.5624</v>
+        <v>72.5806</v>
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
+          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
       <c r="I44" s="8" t="inlineStr">
         <is>
-          <t>2026-09-05 08:40:34 UTC</t>
+          <t>2026-09-09 05:26:21 UTC</t>
         </is>
       </c>
       <c r="J44" s="8" t="n">
-        <v>4280</v>
+        <v>0</v>
       </c>
       <c r="K44" s="8" t="inlineStr">
         <is>
-          <t>cam04-p1-t3</t>
+          <t>cam01-GJ01KA7392-0</t>
         </is>
       </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>/evidence/cam04_GJ01AB1234_20260905_103244_788186.jpg</t>
+          <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
       <c r="M44" s="8" t="inlineStr">
@@ -3224,54 +3224,54 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>GJ18CD5678</t>
+          <t>GJ03CJ6081</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>97.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>cam04</t>
+          <t>cam17</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>04 Paldi Circle</t>
+          <t>17 Rajkot Bus Port CCTV</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Traffic Police</t>
+          <t>Municipal Corporation</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>23.0104</v>
+        <v>22.217</v>
       </c>
       <c r="G45" t="n">
-        <v>72.5624</v>
+        <v>70.79000000000001</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
+          <t>Rajkot Bus Port, Rajkot</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-05 08:40:34 UTC</t>
+          <t>2026-09-09 05:26:21 UTC</t>
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8720</v>
+        <v>0</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>cam04-p1-t4</t>
+          <t>cam17-GJ03CJ6081-0</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>/evidence/cam04_GJ18CD5678_20260905_103310_149966.jpg</t>
+          <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3280,1070 +3280,8 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>GJ05JV7219</t>
-        </is>
-      </c>
-      <c r="B46" s="8" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>cam04</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>04 Paldi Circle</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F46" s="8" t="n">
-        <v>23.0104</v>
-      </c>
-      <c r="G46" s="8" t="n">
-        <v>72.5624</v>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I46" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:40:34 UTC</t>
-        </is>
-      </c>
-      <c r="J46" s="8" t="n">
-        <v>13160</v>
-      </c>
-      <c r="K46" s="8" t="inlineStr">
-        <is>
-          <t>cam04-p1-t5</t>
-        </is>
-      </c>
-      <c r="L46" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam04_GJ05JV7219_20260905_103333_432433.jpg</t>
-        </is>
-      </c>
-      <c r="M46" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>MH12DE1433</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>97.3</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>cam04</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>04 Paldi Circle</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>23.0104</v>
-      </c>
-      <c r="G47" t="n">
-        <v>72.5624</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:40:34 UTC</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>17480</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>cam04-p1-t6</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>/evidence/cam04_MH12DE1433_20260905_103354_883370.jpg</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>RJ14GH9012</t>
-        </is>
-      </c>
-      <c r="B48" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>cam04</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>04 Paldi Circle</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F48" s="8" t="n">
-        <v>23.0104</v>
-      </c>
-      <c r="G48" s="8" t="n">
-        <v>72.5624</v>
-      </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I48" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:40:34 UTC</t>
-        </is>
-      </c>
-      <c r="J48" s="8" t="n">
-        <v>21920</v>
-      </c>
-      <c r="K48" s="8" t="inlineStr">
-        <is>
-          <t>cam04-p1-t8</t>
-        </is>
-      </c>
-      <c r="L48" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam04_RJ14GH9012_20260905_103416_725146.jpg</t>
-        </is>
-      </c>
-      <c r="M48" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>GJ27XY4455</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>cam04</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>04 Paldi Circle</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F49" t="n">
-        <v>23.0104</v>
-      </c>
-      <c r="G49" t="n">
-        <v>72.5624</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Paldi Circle, Paldi, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:40:34 UTC</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>26360</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>cam04-p1-t9</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>/evidence/cam04_GJ27XY4455_20260905_103429_576600.jpg</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>GJ01AB1234</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F50" s="8" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G50" s="8" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H50" s="8" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I50" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J50" s="8" t="n">
-        <v>1040</v>
-      </c>
-      <c r="K50" s="8" t="inlineStr">
-        <is>
-          <t>cam14-p1-t2</t>
-        </is>
-      </c>
-      <c r="L50" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_GJ01AB1234_20260905_102954_387864.jpg</t>
-        </is>
-      </c>
-      <c r="M50" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>GJ01AB1234</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>100</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G51" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J51" t="n">
-        <v>4280</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>cam14-p1-t3</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_GJ01AB1234_20260905_103012_087080.jpg</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>GJ18CD5678</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F52" s="8" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G52" s="8" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H52" s="8" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I52" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J52" s="8" t="n">
-        <v>8720</v>
-      </c>
-      <c r="K52" s="8" t="inlineStr">
-        <is>
-          <t>cam14-p1-t4</t>
-        </is>
-      </c>
-      <c r="L52" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_GJ18CD5678_20260905_103036_123637.jpg</t>
-        </is>
-      </c>
-      <c r="M52" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>GJ05JV7219</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G53" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J53" t="n">
-        <v>13160</v>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>cam14-p1-t5</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_GJ05JV7219_20260905_103100_387510.jpg</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>MH12DE1433</t>
-        </is>
-      </c>
-      <c r="B54" s="8" t="n">
-        <v>97.3</v>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G54" s="8" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H54" s="8" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I54" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J54" s="8" t="n">
-        <v>17480</v>
-      </c>
-      <c r="K54" s="8" t="inlineStr">
-        <is>
-          <t>cam14-p1-t6</t>
-        </is>
-      </c>
-      <c r="L54" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_MH12DE1433_20260905_103122_464237.jpg</t>
-        </is>
-      </c>
-      <c r="M54" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>RJ14GH9012</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>100</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G55" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J55" t="n">
-        <v>21920</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>cam14-p1-t8</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_RJ14GH9012_20260905_103145_899297.jpg</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>GJ27XY4455</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
-        <is>
-          <t>cam14</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>14 Delight RLVD</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F56" s="8" t="n">
-        <v>23.047</v>
-      </c>
-      <c r="G56" s="8" t="n">
-        <v>72.58799999999999</v>
-      </c>
-      <c r="H56" s="8" t="inlineStr">
-        <is>
-          <t>Delight Red Light Violation Detection, Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I56" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:32:34 UTC</t>
-        </is>
-      </c>
-      <c r="J56" s="8" t="n">
-        <v>26360</v>
-      </c>
-      <c r="K56" s="8" t="inlineStr">
-        <is>
-          <t>cam14-p1-t9</t>
-        </is>
-      </c>
-      <c r="L56" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam14_GJ27XY4455_20260905_103159_617749.jpg</t>
-        </is>
-      </c>
-      <c r="M56" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>GJ01AB1234</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G57" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J57" t="n">
-        <v>1040</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>cam01-p1-t2</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_GJ01AB1234_20260905_102656_934184.jpg</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>GJ01AB1234</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C58" s="8" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F58" s="8" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G58" s="8" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H58" s="8" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I58" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J58" s="8" t="n">
-        <v>4280</v>
-      </c>
-      <c r="K58" s="8" t="inlineStr">
-        <is>
-          <t>cam01-p1-t3</t>
-        </is>
-      </c>
-      <c r="L58" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_GJ01AB1234_20260905_102742_614073.jpg</t>
-        </is>
-      </c>
-      <c r="M58" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>GJ18CD5678</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G59" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J59" t="n">
-        <v>8720</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>cam01-p1-t4</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_GJ18CD5678_20260905_102810_695990.jpg</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>GJ05JV7219</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="C60" s="8" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D60" s="8" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E60" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F60" s="8" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G60" s="8" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H60" s="8" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J60" s="8" t="n">
-        <v>13160</v>
-      </c>
-      <c r="K60" s="8" t="inlineStr">
-        <is>
-          <t>cam01-p1-t5</t>
-        </is>
-      </c>
-      <c r="L60" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_GJ05JV7219_20260905_102833_792575.jpg</t>
-        </is>
-      </c>
-      <c r="M60" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>MH12DE1433</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>97.3</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G61" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J61" t="n">
-        <v>17480</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>cam01-p1-t6</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_MH12DE1433_20260905_102853_408705.jpg</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>RJ14GH9012</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D62" s="8" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E62" s="8" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F62" s="8" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G62" s="8" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H62" s="8" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I62" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J62" s="8" t="n">
-        <v>21920</v>
-      </c>
-      <c r="K62" s="8" t="inlineStr">
-        <is>
-          <t>cam01-p1-t8</t>
-        </is>
-      </c>
-      <c r="L62" s="8" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_RJ14GH9012_20260905_102914_493099.jpg</t>
-        </is>
-      </c>
-      <c r="M62" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>GJ27XY4455</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>cam01</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>01 Chiman bhai Bridge</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Traffic Police</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>23.0587</v>
-      </c>
-      <c r="G63" t="n">
-        <v>72.5806</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>2026-09-05 08:26:34 UTC</t>
-        </is>
-      </c>
-      <c r="J63" t="n">
-        <v>26360</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>cam01-p1-t9</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>/evidence/cam01_GJ27XY4455_20260905_102926_716445.jpg</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M63"/>
+  <autoFilter ref="A1:M45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(submission): polish sentinel_output_report.xlsx formatting and remove corrupted unicode characters
</commit_message>
<xml_diff>
--- a/submission/sentinel_output_report.xlsx
+++ b/submission/sentinel_output_report.xlsx
@@ -19,8 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,24 +32,55 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="001A2332"/>
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00555555"/>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="004A5568"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="002D3748"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001A202C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001A2332"/>
       <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
+      <name val="Segoe UI"/>
+      <color rgb="004A5568"/>
+      <sz val="9"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001A202C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002D3748"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -63,11 +97,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5FA"/>
+        <fgColor rgb="00F4F7FA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,24 +109,73 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,136 +541,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sentinel — ANPR Output Report</t>
+          <t>Sentinel - ANPR Output Report</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gujarat CCTV Integration Hackathon 2026 · Model 1 + Model 2</t>
+          <t>Gujarat CCTV Integration Hackathon 2026 | Track: Model 1 + Model 2 | Team: KodeMatrix</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Generated (UTC)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-11 09:38:27</t>
+          <t>Team Name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>KodeMatrix</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Data source</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sentinel sandbox grid (cctv.corp8.cloud)</t>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/DevamShah1211/Sentinel-Hackathone</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Reporting window</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>all indexed detections</t>
+          <t>Generated (UTC)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 09:38:27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Total detections</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>44</v>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Sentinel sandbox grid (cctv.corp8.cloud)</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Unique plates</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>8</v>
+          <t>Reporting window</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>all indexed detections</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cameras covered</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>12</v>
+          <t>Total detections</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>Unique plates</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Cameras covered</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Watchlist alerts</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" s="4" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Method and limitations</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>• Plates are read by pretrained open-source models (YOLOv9 plate detector, cct-s-v2 OCR) running locally on CPU. No video frame leaves the deployment and no external API is used in the detection or alerting path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>• Each row is one vehicle pass, not one frame: reads are aggregated across a vehicle's track by confidence-weighted per-character voting, then validated against Indian plate grammar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>• The sandbox catalogue publishes only camera id and name. Coordinates are resolved by hand-verification or OpenStreetMap geocoding and each camera records which method was used; they are approximate site locations, not a surveyed asset register.</t>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>- Plates are read by pretrained open-source models (YOLOv9 plate detector, cct-s-v2 OCR) running locally on CPU. No video frame leaves the deployment and no external API is used in the detection or alerting path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>- Each row is one vehicle pass, not one frame: reads are aggregated across a vehicle's track by confidence-weighted per-character voting, then validated against Indian plate grammar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>- The sandbox catalogue publishes only camera id and name. Coordinates are resolved by hand-verification or OpenStreetMap geocoding and each camera records which method was used; they are approximate site locations, not a surveyed asset register.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -603,2678 +710,2678 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="54" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Plate</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Confidence %</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Camera ID</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Camera Name</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Detected At (UTC)</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Stream PTS (ms)</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Track ID</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Evidence Crop</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Location Source</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="12" t="n">
         <v>23.035</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="12" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 05:42:50 UTC</t>
         </is>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>cam13-GJ03CJ6081-2</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="15" t="n">
         <v>96</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="18" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="18" t="n">
         <v>72.581</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:58:50 UTC</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>cam12-GJ18DH2745-3</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>cam03</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>03 O.N.G.C. Office</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="12" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="12" t="n">
         <v>72.53100000000001</v>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>ONGC Office, Chandkheda, Ahmedabad</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:54:50 UTC</t>
         </is>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>cam03-MH12QP5837-3</t>
         </is>
       </c>
-      <c r="L4" s="8" t="inlineStr">
+      <c r="L4" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>cam01</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="18" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="18" t="n">
         <v>72.5806</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:43:50 UTC</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>cam01-RJ14SL3926-2</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="M5" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>cam02</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>02 Janpath</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="12" t="n">
         <v>23.0299</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="12" t="n">
         <v>72.57129999999999</v>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:41:50 UTC</t>
         </is>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="13" t="n">
         <v>4000</v>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>cam02-GJ01KA7392-4</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="15" t="n">
         <v>96</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="18" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="18" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:40:50 UTC</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>cam05-GJ18DH2745-2</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>cam14</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>14 Delight RLVD</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="12" t="n">
         <v>23.047</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="12" t="n">
         <v>72.58799999999999</v>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:36:50 UTC</t>
         </is>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>cam14-MH12QP5837-2</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="15" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="18" t="n">
         <v>23.035</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="18" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:33:50 UTC</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>cam13-GJ01KA7392-3</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="F10" s="12" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="12" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:31:50 UTC</t>
         </is>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K10" s="8" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>cam05-RJ14SL3926-1</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="18" t="n">
         <v>23.035</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="18" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:25:50 UTC</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>cam13-MH12QP5837-1</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>cam18</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>18 Rajkot CCTV</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F12" s="8" t="n">
+      <c r="F12" s="12" t="n">
         <v>22.3039</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="12" t="n">
         <v>70.8022</v>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Rajkot City Surveillance</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:25:50 UTC</t>
         </is>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K12" s="8" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>cam18-GJ03CJ6081-1</t>
         </is>
       </c>
-      <c r="L12" s="8" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="15" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>cam04</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>04 Paldi Circle</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="18" t="n">
         <v>23.0104</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="18" t="n">
         <v>72.5624</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:24:50 UTC</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>cam04-GJ01KA7392-2</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>GJ27BG4108</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="12" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="12" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:21:50 UTC</t>
         </is>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>cam05-GJ27BG4108-1</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam16_GJ27BG4108_20260911_060753_475745.jpg</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="15" t="n">
         <v>96</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>cam02</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>02 Janpath</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="18" t="n">
         <v>23.0299</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="18" t="n">
         <v>72.57129999999999</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:21:50 UTC</t>
         </is>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>cam02-GJ18DH2745-1</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L15" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>GJ27BG4108</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>cam16</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>16 Visat P2</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="F16" s="12" t="n">
         <v>23.101</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="12" t="n">
         <v>72.583</v>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>Visat Point 2, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:19:50 UTC</t>
         </is>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J16" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="8" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>cam16-GJ27BG4108-0</t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr">
+      <c r="L16" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam16_GJ27BG4108_20260911_060753_475745.jpg</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="15" t="n">
         <v>96</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>cam04</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>04 Paldi Circle</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="18" t="n">
         <v>23.0104</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="18" t="n">
         <v>72.5624</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:15:50 UTC</t>
         </is>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>cam04-GJ18DH2745-0</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260911_060752_391724.jpg</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>cam14</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>14 Delight RLVD</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="F18" s="12" t="n">
         <v>23.047</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="12" t="n">
         <v>72.58799999999999</v>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:12:50 UTC</t>
         </is>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J18" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K18" s="8" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>cam14-GJ01KA7392-1</t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
+      <c r="L18" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
-      <c r="M18" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="18" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="18" t="n">
         <v>72.581</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:12:50 UTC</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>cam12-RJ14SL3926-0</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260911_060753_741893.jpg</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="9" t="n">
         <v>97</v>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>cam15</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>15 Suvidha park</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="F20" s="12" t="n">
         <v>23.081</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="12" t="n">
         <v>72.529</v>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>Suvidha Park, Ahmedabad</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:10:50 UTC</t>
         </is>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>cam15-MH12QP5837-0</t>
         </is>
       </c>
-      <c r="L20" s="8" t="inlineStr">
+      <c r="L20" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260911_060752_994735.jpg</t>
         </is>
       </c>
-      <c r="M20" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>cam17</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>17 Rajkot Bus Port CCTV</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>Municipal Corporation</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="18" t="n">
         <v>22.217</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="18" t="n">
         <v>70.79000000000001</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>Rajkot Bus Port, Rajkot</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>2026-09-11 04:07:50 UTC</t>
         </is>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>cam17-GJ03CJ6081-0</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260911_060751_829832.jpg</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>cam01</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="12" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="12" t="n">
         <v>72.5806</v>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>2026-09-11 04:07:50 UTC</t>
         </is>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J22" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="8" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>cam01-GJ01KA7392-0</t>
         </is>
       </c>
-      <c r="L22" s="8" t="inlineStr">
+      <c r="L22" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260911_060751_033936.jpg</t>
         </is>
       </c>
-      <c r="M22" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>RJ4E4555</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="15" t="n">
         <v>78.5</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="18" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="18" t="n">
         <v>72.581</v>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="17" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 11:16:42 UTC</t>
         </is>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="19" t="n">
         <v>7150</v>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>cam12-t2</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ4E4555_20260909_111641_637598.jpg</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>RJ3E4555</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="9" t="n">
         <v>80.5</v>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="12" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="12" t="n">
         <v>72.581</v>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="I24" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 11:16:15 UTC</t>
         </is>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J24" s="13" t="n">
         <v>2150</v>
       </c>
-      <c r="K24" s="8" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>cam12-t1</t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
+      <c r="L24" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ3E4555_20260909_111614_390210.jpg</t>
         </is>
       </c>
-      <c r="M24" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="M24" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="18" t="n">
         <v>23.035</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="18" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 07:01:21 UTC</t>
         </is>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="K25" s="17" t="inlineStr">
         <is>
           <t>cam13-GJ03CJ6081-2</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="L25" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F26" s="8" t="n">
+      <c r="F26" s="12" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="12" t="n">
         <v>72.581</v>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I26" s="8" t="inlineStr">
+      <c r="I26" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 06:17:21 UTC</t>
         </is>
       </c>
-      <c r="J26" s="8" t="n">
+      <c r="J26" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="K26" s="8" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>cam12-GJ18DH2745-3</t>
         </is>
       </c>
-      <c r="L26" s="8" t="inlineStr">
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
-      <c r="M26" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="M26" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>cam03</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>03 O.N.G.C. Office</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="18" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" s="18" t="n">
         <v>72.53100000000001</v>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>ONGC Office, Chandkheda, Ahmedabad</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 06:13:21 UTC</t>
         </is>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" s="19" t="n">
         <v>3000</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="17" t="inlineStr">
         <is>
           <t>cam03-MH12QP5837-3</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>cam01</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="12" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="12" t="n">
         <v>72.5806</v>
       </c>
-      <c r="H28" s="8" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
-      <c r="I28" s="8" t="inlineStr">
+      <c r="I28" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 06:02:21 UTC</t>
         </is>
       </c>
-      <c r="J28" s="8" t="n">
+      <c r="J28" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K28" s="8" t="inlineStr">
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>cam01-RJ14SL3926-2</t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
+      <c r="L28" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
-      <c r="M28" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="M28" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="15" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>cam02</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>02 Janpath</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="18" t="n">
         <v>23.0299</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" s="18" t="n">
         <v>72.57129999999999</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="17" t="inlineStr">
         <is>
           <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 06:00:21 UTC</t>
         </is>
       </c>
-      <c r="J29" t="n">
+      <c r="J29" s="19" t="n">
         <v>4000</v>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="17" t="inlineStr">
         <is>
           <t>cam02-GJ01KA7392-4</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="12" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="12" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I30" s="8" t="inlineStr">
+      <c r="I30" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:59:21 UTC</t>
         </is>
       </c>
-      <c r="J30" s="8" t="n">
+      <c r="J30" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K30" s="8" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>cam05-GJ18DH2745-2</t>
         </is>
       </c>
-      <c r="L30" s="8" t="inlineStr">
+      <c r="L30" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
-      <c r="M30" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="M30" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>cam14</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>14 Delight RLVD</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F31" s="18" t="n">
         <v>23.047</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" s="18" t="n">
         <v>72.58799999999999</v>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="17" t="inlineStr">
         <is>
           <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:55:21 UTC</t>
         </is>
       </c>
-      <c r="J31" t="n">
+      <c r="J31" s="19" t="n">
         <v>2000</v>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="17" t="inlineStr">
         <is>
           <t>cam14-MH12QP5837-2</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="12" t="n">
         <v>23.035</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="12" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I32" s="8" t="inlineStr">
+      <c r="I32" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:52:21 UTC</t>
         </is>
       </c>
-      <c r="J32" s="8" t="n">
+      <c r="J32" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="K32" s="8" t="inlineStr">
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>cam13-GJ01KA7392-3</t>
         </is>
       </c>
-      <c r="L32" s="8" t="inlineStr">
+      <c r="L32" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
-      <c r="M32" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="M32" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="18" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" s="18" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:50:21 UTC</t>
         </is>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="17" t="inlineStr">
         <is>
           <t>cam05-RJ14SL3926-1</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>cam18</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>18 Rajkot CCTV</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="12" t="n">
         <v>22.3039</v>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="12" t="n">
         <v>70.8022</v>
       </c>
-      <c r="H34" s="8" t="inlineStr">
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>Rajkot City Surveillance</t>
         </is>
       </c>
-      <c r="I34" s="8" t="inlineStr">
+      <c r="I34" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:44:21 UTC</t>
         </is>
       </c>
-      <c r="J34" s="8" t="n">
+      <c r="J34" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K34" s="8" t="inlineStr">
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>cam18-GJ03CJ6081-1</t>
         </is>
       </c>
-      <c r="L34" s="8" t="inlineStr">
+      <c r="L34" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
-      <c r="M34" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="M34" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>cam13</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>13 CN Vidhyalaya</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F35" t="n">
+      <c r="F35" s="18" t="n">
         <v>23.035</v>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" s="18" t="n">
         <v>72.54900000000001</v>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="17" t="inlineStr">
         <is>
           <t>C N Vidyalaya, Ambawadi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:44:21 UTC</t>
         </is>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="17" t="inlineStr">
         <is>
           <t>cam13-MH12QP5837-1</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>cam04</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>04 Paldi Circle</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="12" t="n">
         <v>23.0104</v>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="12" t="n">
         <v>72.5624</v>
       </c>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr">
         <is>
           <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I36" s="8" t="inlineStr">
+      <c r="I36" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:43:21 UTC</t>
         </is>
       </c>
-      <c r="J36" s="8" t="n">
+      <c r="J36" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="K36" s="8" t="inlineStr">
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>cam04-GJ01KA7392-2</t>
         </is>
       </c>
-      <c r="L36" s="8" t="inlineStr">
+      <c r="L36" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
-      <c r="M36" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="M36" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>GJ27BG4108</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>cam05</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>05 Visat teen Rasta</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="F37" s="18" t="n">
         <v>23.0999</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G37" s="18" t="n">
         <v>72.5814</v>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" s="17" t="inlineStr">
         <is>
           <t>Visat Teen Rasta, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:40:21 UTC</t>
         </is>
       </c>
-      <c r="J37" t="n">
+      <c r="J37" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K37" s="17" t="inlineStr">
         <is>
           <t>cam05-GJ27BG4108-1</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L37" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam16_GJ27BG4108_20260909_072626_710757.jpg</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B38" s="8" t="n">
+      <c r="B38" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>cam02</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>02 Janpath</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="12" t="n">
         <v>23.0299</v>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="12" t="n">
         <v>72.57129999999999</v>
       </c>
-      <c r="H38" s="8" t="inlineStr">
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>Janpath, Ashram Road, Ahmedabad</t>
         </is>
       </c>
-      <c r="I38" s="8" t="inlineStr">
+      <c r="I38" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:40:21 UTC</t>
         </is>
       </c>
-      <c r="J38" s="8" t="n">
+      <c r="J38" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="K38" s="8" t="inlineStr">
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>cam02-GJ18DH2745-1</t>
         </is>
       </c>
-      <c r="L38" s="8" t="inlineStr">
+      <c r="L38" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
-      <c r="M38" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="M38" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>GJ27BG4108</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="16" t="inlineStr">
         <is>
           <t>cam16</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>16 Visat P2</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="18" t="n">
         <v>23.101</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" s="18" t="n">
         <v>72.583</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" s="17" t="inlineStr">
         <is>
           <t>Visat Point 2, Sabarmati, Ahmedabad</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:38:21 UTC</t>
         </is>
       </c>
-      <c r="J39" t="n">
+      <c r="J39" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="17" t="inlineStr">
         <is>
           <t>cam16-GJ27BG4108-0</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam16_GJ27BG4108_20260909_072626_710757.jpg</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>GJ18DH2745</t>
         </is>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>cam04</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>04 Paldi Circle</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="12" t="n">
         <v>23.0104</v>
       </c>
-      <c r="G40" s="8" t="n">
+      <c r="G40" s="12" t="n">
         <v>72.5624</v>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="H40" s="11" t="inlineStr">
         <is>
           <t>Paldi Circle, Paldi, Ahmedabad</t>
         </is>
       </c>
-      <c r="I40" s="8" t="inlineStr">
+      <c r="I40" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:34:21 UTC</t>
         </is>
       </c>
-      <c r="J40" s="8" t="n">
+      <c r="J40" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K40" s="8" t="inlineStr">
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>cam04-GJ18DH2745-0</t>
         </is>
       </c>
-      <c r="L40" s="8" t="inlineStr">
+      <c r="L40" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam04_GJ18DH2745_20260909_072624_696402.jpg</t>
         </is>
       </c>
-      <c r="M40" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="M40" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="15" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="16" t="inlineStr">
         <is>
           <t>cam14</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>14 Delight RLVD</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="18" t="n">
         <v>23.047</v>
       </c>
-      <c r="G41" t="n">
+      <c r="G41" s="18" t="n">
         <v>72.58799999999999</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="17" t="inlineStr">
         <is>
           <t>Delight Red Light Violation Detection, Ahmedabad</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:31:21 UTC</t>
         </is>
       </c>
-      <c r="J41" t="n">
+      <c r="J41" s="19" t="n">
         <v>1000</v>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="17" t="inlineStr">
         <is>
           <t>cam14-GJ01KA7392-1</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>RJ14SL3926</t>
         </is>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>cam12</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>12 Tri Mandir Adalaj Tollnaka</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="12" t="n">
         <v>23.1645</v>
       </c>
-      <c r="G42" s="8" t="n">
+      <c r="G42" s="12" t="n">
         <v>72.581</v>
       </c>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="H42" s="11" t="inlineStr">
         <is>
           <t>Tri Mandir, Adalaj Toll Naka</t>
         </is>
       </c>
-      <c r="I42" s="8" t="inlineStr">
+      <c r="I42" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:31:21 UTC</t>
         </is>
       </c>
-      <c r="J42" s="8" t="n">
+      <c r="J42" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K42" s="8" t="inlineStr">
+      <c r="K42" s="11" t="inlineStr">
         <is>
           <t>cam12-RJ14SL3926-0</t>
         </is>
       </c>
-      <c r="L42" s="8" t="inlineStr">
+      <c r="L42" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam12_RJ14SL3926_20260909_072627_326850.jpg</t>
         </is>
       </c>
-      <c r="M42" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="M42" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>MH12QP5837</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="16" t="inlineStr">
         <is>
           <t>cam15</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>15 Suvidha park</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>City Surveillance</t>
         </is>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="18" t="n">
         <v>23.081</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="18" t="n">
         <v>72.529</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="17" t="inlineStr">
         <is>
           <t>Suvidha Park, Ahmedabad</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:29:21 UTC</t>
         </is>
       </c>
-      <c r="J43" t="n">
+      <c r="J43" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="17" t="inlineStr">
         <is>
           <t>cam15-MH12QP5837-0</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam15_MH12QP5837_20260909_072625_641255.jpg</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>GJ01KA7392</t>
         </is>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="9" t="n">
         <v>97.09999999999999</v>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>cam01</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
+      <c r="D44" s="11" t="inlineStr">
         <is>
           <t>01 Chiman bhai Bridge</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Traffic Police</t>
         </is>
       </c>
-      <c r="F44" s="8" t="n">
+      <c r="F44" s="12" t="n">
         <v>23.0587</v>
       </c>
-      <c r="G44" s="8" t="n">
+      <c r="G44" s="12" t="n">
         <v>72.5806</v>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="H44" s="11" t="inlineStr">
         <is>
           <t>Chimanbhai Patel Bridge (Subhash Bridge), Ahmedabad</t>
         </is>
       </c>
-      <c r="I44" s="8" t="inlineStr">
+      <c r="I44" s="10" t="inlineStr">
         <is>
           <t>2026-09-09 05:26:21 UTC</t>
         </is>
       </c>
-      <c r="J44" s="8" t="n">
+      <c r="J44" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K44" s="8" t="inlineStr">
+      <c r="K44" s="11" t="inlineStr">
         <is>
           <t>cam01-GJ01KA7392-0</t>
         </is>
       </c>
-      <c r="L44" s="8" t="inlineStr">
+      <c r="L44" s="11" t="inlineStr">
         <is>
           <t>/evidence/cam01_GJ01KA7392_20260909_072622_524948.jpg</t>
         </is>
       </c>
-      <c r="M44" s="8" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="M44" s="10" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>GJ03CJ6081</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="16" t="inlineStr">
         <is>
           <t>cam17</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>17 Rajkot Bus Port CCTV</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="17" t="inlineStr">
         <is>
           <t>Municipal Corporation</t>
         </is>
       </c>
-      <c r="F45" t="n">
+      <c r="F45" s="18" t="n">
         <v>22.217</v>
       </c>
-      <c r="G45" t="n">
+      <c r="G45" s="18" t="n">
         <v>70.79000000000001</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="17" t="inlineStr">
         <is>
           <t>Rajkot Bus Port, Rajkot</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="16" t="inlineStr">
         <is>
           <t>2026-09-09 05:26:21 UTC</t>
         </is>
       </c>
-      <c r="J45" t="n">
+      <c r="J45" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="17" t="inlineStr">
         <is>
           <t>cam17-GJ03CJ6081-0</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="17" t="inlineStr">
         <is>
           <t>/evidence/cam17_GJ03CJ6081_20260909_072623_764636.jpg</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M45" s="16" t="inlineStr">
         <is>
           <t>manual</t>
         </is>

</xml_diff>